<commit_message>
enriching controls types description and IPTW choice justification
</commit_message>
<xml_diff>
--- a/results/ate_evalue_survey.xlsx
+++ b/results/ate_evalue_survey.xlsx
@@ -492,13 +492,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.4385066466877225</v>
+        <v>0.4385066466877215</v>
       </c>
       <c r="D2" t="n">
-        <v>1.490394795801431</v>
+        <v>1.49039479580143</v>
       </c>
       <c r="E2" t="n">
-        <v>2.345311079159374</v>
+        <v>2.345311079159371</v>
       </c>
       <c r="F2" t="n">
         <v>2.079226624866933</v>
@@ -514,7 +514,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>3.817947647451507e-21</v>
+        <v>3.817947647451479e-21</v>
       </c>
       <c r="J2" t="b">
         <v>1</v>
@@ -532,13 +532,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>-0.0003080184020601404</v>
+        <v>-0.0003080184020606005</v>
       </c>
       <c r="D3" t="n">
-        <v>1.000280336032678</v>
+        <v>1.000280336032679</v>
       </c>
       <c r="E3" t="n">
-        <v>1.017025921151431</v>
+        <v>1.017025921151445</v>
       </c>
       <c r="F3" t="n">
         <v>1.433204662544642</v>
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>0.9472230553604787</v>
+        <v>0.9472230553604783</v>
       </c>
       <c r="J3" t="b">
         <v>0</v>
@@ -572,13 +572,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.1560165140786414</v>
+        <v>0.1560165140786419</v>
       </c>
       <c r="D4" t="n">
         <v>1.152547866535127</v>
       </c>
       <c r="E4" t="n">
-        <v>1.571855293275395</v>
+        <v>1.571855293275396</v>
       </c>
       <c r="F4" t="n">
         <v>1.381038924028185</v>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>7.251803917655306e-05</v>
+        <v>7.251803917655231e-05</v>
       </c>
       <c r="J4" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Adding notes about descendants (DAG)
</commit_message>
<xml_diff>
--- a/results/ate_evalue_survey.xlsx
+++ b/results/ate_evalue_survey.xlsx
@@ -492,13 +492,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.4385066466877215</v>
+        <v>0.4385066466877225</v>
       </c>
       <c r="D2" t="n">
-        <v>1.49039479580143</v>
+        <v>1.490394795801431</v>
       </c>
       <c r="E2" t="n">
-        <v>2.345311079159371</v>
+        <v>2.345311079159374</v>
       </c>
       <c r="F2" t="n">
         <v>2.079226624866933</v>
@@ -514,7 +514,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>3.817947647451479e-21</v>
+        <v>3.817947647451369e-21</v>
       </c>
       <c r="J2" t="b">
         <v>1</v>
@@ -532,13 +532,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>-0.0003080184020606005</v>
+        <v>-0.0003080184020601404</v>
       </c>
       <c r="D3" t="n">
-        <v>1.000280336032679</v>
+        <v>1.000280336032678</v>
       </c>
       <c r="E3" t="n">
-        <v>1.017025921151445</v>
+        <v>1.017025921151431</v>
       </c>
       <c r="F3" t="n">
         <v>1.433204662544642</v>
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>0.9472230553604783</v>
+        <v>0.9472230553604767</v>
       </c>
       <c r="J3" t="b">
         <v>0</v>
@@ -572,13 +572,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.1560165140786419</v>
+        <v>0.1560165140786423</v>
       </c>
       <c r="D4" t="n">
-        <v>1.152547866535127</v>
+        <v>1.152547866535128</v>
       </c>
       <c r="E4" t="n">
-        <v>1.571855293275396</v>
+        <v>1.571855293275398</v>
       </c>
       <c r="F4" t="n">
         <v>1.381038924028185</v>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>7.251803917655231e-05</v>
+        <v>7.251803917655306e-05</v>
       </c>
       <c r="J4" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
docs(slides): correct sandwich SE explanation in IPTW+GEE deck
</commit_message>
<xml_diff>
--- a/results/ate_evalue_survey.xlsx
+++ b/results/ate_evalue_survey.xlsx
@@ -492,13 +492,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.4731872093428426</v>
+        <v>0.4731872093428416</v>
       </c>
       <c r="D2" t="n">
-        <v>1.538180709341216</v>
+        <v>1.538180709341215</v>
       </c>
       <c r="E2" t="n">
-        <v>2.448026402438805</v>
+        <v>2.448026402438801</v>
       </c>
       <c r="F2" t="n">
         <v>2.182214874657829</v>
@@ -514,7 +514,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>4.491231826565276e-25</v>
+        <v>4.491231826565724e-25</v>
       </c>
       <c r="J2" t="b">
         <v>1</v>
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>0.8572422817678194</v>
+        <v>0.8572422817678176</v>
       </c>
       <c r="J3" t="b">
         <v>0</v>
@@ -572,13 +572,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.163544348696728</v>
+        <v>0.1635443486967275</v>
       </c>
       <c r="D4" t="n">
-        <v>1.160470303859981</v>
+        <v>1.16047030385998</v>
       </c>
       <c r="E4" t="n">
-        <v>1.592003642410892</v>
+        <v>1.59200364241089</v>
       </c>
       <c r="F4" t="n">
         <v>1.383351419900095</v>

</xml_diff>